<commit_message>
Suppressed Session Warnings and Added Login Preference Cookie Management
Suppressed session warnings with @ operator in session_start() calls to prevent errors during concurrent test runs. Added guard to only regenerate session ID when session is active. Implemented login preference cookie that remembers user's choice between Google and email sign-in for 30 days - cookie is set after successful email/2FA login and cleared when signing in with Google to prevent auto-expansion of email section. Adde
</commit_message>
<xml_diff>
--- a/documentation/Issue Tracker.xlsx
+++ b/documentation/Issue Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAMP\htdocs\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827AA061-F478-4499-BA54-6E844FA6F724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADDE166-48A9-47D4-8EA1-6DEA16EDD5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B30AA0F8-B590-4D13-9530-2CA817625601}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="284">
   <si>
     <t>ISSUE TRACKER</t>
   </si>
@@ -892,6 +892,9 @@
   </si>
   <si>
     <t>Retest</t>
+  </si>
+  <si>
+    <t>Keeps the login with email section expanded and it's driving me nuts</t>
   </si>
 </sst>
 </file>
@@ -1276,23 +1279,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill>
@@ -1546,6 +1533,14 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <strike val="0"/>
@@ -1650,9 +1645,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="3" xr9:uid="{9287C67C-ECEA-45B3-8051-FC9FD9595AF7}">
-      <tableStyleElement type="wholeTable" dxfId="18"/>
-      <tableStyleElement type="firstRowStripe" dxfId="17"/>
-      <tableStyleElement type="secondRowStripe" dxfId="16"/>
+      <tableStyleElement type="wholeTable" dxfId="17"/>
+      <tableStyleElement type="firstRowStripe" dxfId="16"/>
+      <tableStyleElement type="secondRowStripe" dxfId="15"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1875,21 +1870,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="B13:J247" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B14:J247">
-    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="1"/>
+    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="12"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2298,24 +2293,24 @@
         <v>9</v>
       </c>
       <c r="F6" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E6),"")</f>
-        <v>46</v>
+        <f t="shared" ref="F6:H9" si="0">IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E6),"")</f>
+        <v>52</v>
       </c>
       <c r="G6" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,G$5,$H$14:$H$247,$E6),"")</f>
-        <v>85</v>
+        <f t="shared" si="0"/>
+        <v>92</v>
       </c>
       <c r="H6" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,H$5,$H$14:$H$247,$E6),"")</f>
-        <v>31</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
       <c r="I6" s="16">
         <f>IFERROR(SUM(F6:H6),"-")</f>
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="J6" s="17">
         <f>IFERROR(I6/$I$10,"-")</f>
-        <v>0.9050279329608939</v>
+        <v>0.98888888888888893</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -2328,15 +2323,15 @@
         <v>11</v>
       </c>
       <c r="F7" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E7),"")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G7" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,G$5,$H$14:$H$247,$E7),"")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H7" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,H$5,$H$14:$H$247,$E7),"")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I7" s="16">
@@ -2356,24 +2351,24 @@
         <v>12</v>
       </c>
       <c r="F8" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E8),"")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G8" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,G$5,$H$14:$H$247,$E8),"")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H8" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,H$5,$H$14:$H$247,$E8),"")</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="I8" s="16">
         <f>IFERROR(SUM(F8:H8),"-")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="17">
         <f>IFERROR(I8/$I$10,"-")</f>
-        <v>0</v>
+        <v>5.5555555555555558E-3</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
@@ -2384,24 +2379,24 @@
         <v>282</v>
       </c>
       <c r="F9" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E9),"")</f>
-        <v>6</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="G9" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,G$5,$H$14:$H$247,$E9),"")</f>
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="H9" s="27">
-        <f>IFERROR(COUNTIFS($E$14:$E$247,H$5,$H$14:$H$247,$E9),"")</f>
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="I9" s="16">
         <f>IFERROR(SUM(F9:H9),"-")</f>
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="J9" s="17">
         <f>IFERROR(I9/$I$10,"-")</f>
-        <v>9.4972067039106142E-2</v>
+        <v>5.5555555555555558E-3</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
@@ -2423,11 +2418,11 @@
       </c>
       <c r="H10" s="16">
         <f>IFERROR(SUM(H6:H9),"-")</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I10" s="16">
         <f>IFERROR(SUM(F10:H10),"-")</f>
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J10" s="18"/>
     </row>
@@ -2442,15 +2437,15 @@
       </c>
       <c r="F11" s="17">
         <f>IFERROR(F10/$I$10,"-")</f>
-        <v>0.29050279329608941</v>
+        <v>0.28888888888888886</v>
       </c>
       <c r="G11" s="17">
-        <f t="shared" ref="G11:H11" si="0">IFERROR(G10/$I$10,"-")</f>
-        <v>0.51955307262569828</v>
+        <f t="shared" ref="G11:H11" si="1">IFERROR(G10/$I$10,"-")</f>
+        <v>0.51666666666666672</v>
       </c>
       <c r="H11" s="17">
-        <f t="shared" si="0"/>
-        <v>0.18994413407821228</v>
+        <f t="shared" si="1"/>
+        <v>0.19444444444444445</v>
       </c>
       <c r="I11" s="18"/>
       <c r="J11" s="19"/>
@@ -2511,7 +2506,7 @@
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I14" s="25"/>
       <c r="J14" s="25"/>
@@ -2553,7 +2548,7 @@
       <c r="F16" s="24"/>
       <c r="G16" s="24"/>
       <c r="H16" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I16" s="25"/>
       <c r="J16" s="25"/>
@@ -2574,7 +2569,7 @@
       <c r="F17" s="24"/>
       <c r="G17" s="24"/>
       <c r="H17" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I17" s="25"/>
       <c r="J17" s="25"/>
@@ -2595,7 +2590,7 @@
       <c r="F18" s="24"/>
       <c r="G18" s="24"/>
       <c r="H18" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I18" s="25"/>
       <c r="J18" s="25"/>
@@ -2616,7 +2611,7 @@
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
       <c r="H19" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I19" s="25"/>
       <c r="J19" s="25"/>
@@ -2637,7 +2632,7 @@
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
       <c r="H20" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
@@ -2658,7 +2653,7 @@
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
       <c r="H21" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I21" s="25"/>
       <c r="J21" s="25"/>
@@ -2679,7 +2674,7 @@
       <c r="F22" s="24"/>
       <c r="G22" s="24"/>
       <c r="H22" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I22" s="25"/>
       <c r="J22" s="25"/>
@@ -2700,7 +2695,7 @@
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I23" s="25"/>
       <c r="J23" s="25"/>
@@ -2721,7 +2716,7 @@
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
       <c r="H24" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I24" s="25"/>
       <c r="J24" s="25"/>
@@ -2742,7 +2737,7 @@
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
       <c r="H25" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I25" s="25"/>
       <c r="J25" s="25"/>
@@ -2763,7 +2758,7 @@
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
       <c r="H26" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I26" s="25"/>
       <c r="J26" s="25"/>
@@ -2784,7 +2779,7 @@
       <c r="F27" s="24"/>
       <c r="G27" s="24"/>
       <c r="H27" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I27" s="25"/>
       <c r="J27" s="25"/>
@@ -2805,7 +2800,7 @@
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I28" s="25"/>
       <c r="J28" s="25"/>
@@ -2826,7 +2821,7 @@
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I29" s="25"/>
       <c r="J29" s="25"/>
@@ -2847,7 +2842,7 @@
       <c r="F30" s="24"/>
       <c r="G30" s="24"/>
       <c r="H30" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I30" s="25"/>
       <c r="J30" s="25"/>
@@ -6276,13 +6271,23 @@
       <c r="J193" s="25"/>
     </row>
     <row r="194" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B194" s="21"/>
-      <c r="C194" s="22"/>
-      <c r="D194" s="23"/>
-      <c r="E194" s="24"/>
+      <c r="B194" s="21">
+        <v>180</v>
+      </c>
+      <c r="C194" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D194" s="23" t="s">
+        <v>283</v>
+      </c>
+      <c r="E194" s="24" t="s">
+        <v>5</v>
+      </c>
       <c r="F194" s="24"/>
       <c r="G194" s="24"/>
-      <c r="H194" s="24"/>
+      <c r="H194" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I194" s="25"/>
       <c r="J194" s="25"/>
     </row>
@@ -6888,21 +6893,18 @@
     <mergeCell ref="B8:B9"/>
   </mergeCells>
   <conditionalFormatting sqref="B13:J247">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$H13="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$H13="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$H13="Retest"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select a status from the list." sqref="H194:H247" xr:uid="{51942771-9FE5-4FA9-93D4-101C615BE219}">
-      <formula1>$E$6:$E$8</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H13:H193" xr:uid="{BC7A51A1-A261-4287-90BE-9E44AA681871}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H13 H14:H247" xr:uid="{BC7A51A1-A261-4287-90BE-9E44AA681871}">
       <formula1>$E$6:$E$9</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select a priority level from the list." sqref="E14:E247" xr:uid="{25B8D43A-C4E7-4DCD-9407-5BDDB17BFA14}">

</xml_diff>

<commit_message>
Refactored Remember Me System to Use Signed Cookies Instead of Database Tokens
Replaced database-backed remember me tokens with simpler signed cookie approach using HMAC signatures. Changed token format from selector:token to userId:expiry:signature for stateless validation. Removed database lookups and token storage - validation now only verifies signature and checks user exists. Added backwards compatibility for legacy database tokens. Fixed remember me auto-login timing by moving attemptRememberMeLogin() call
</commit_message>
<xml_diff>
--- a/documentation/Issue Tracker.xlsx
+++ b/documentation/Issue Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAMP\htdocs\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADDE166-48A9-47D4-8EA1-6DEA16EDD5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCB103E-706F-437F-9246-304D43ED5E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B30AA0F8-B590-4D13-9530-2CA817625601}"/>
   </bookViews>
@@ -1279,7 +1279,31 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="20">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1533,14 +1557,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <strike val="0"/>
@@ -1645,9 +1661,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="3" xr9:uid="{9287C67C-ECEA-45B3-8051-FC9FD9595AF7}">
-      <tableStyleElement type="wholeTable" dxfId="17"/>
-      <tableStyleElement type="firstRowStripe" dxfId="16"/>
-      <tableStyleElement type="secondRowStripe" dxfId="15"/>
+      <tableStyleElement type="wholeTable" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="secondRowStripe" dxfId="17"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1870,21 +1886,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="B13:J247" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B14:J247">
-    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="12"/>
+    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="1"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2302,15 +2318,15 @@
       </c>
       <c r="H6" s="27">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="16">
         <f>IFERROR(SUM(F6:H6),"-")</f>
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J6" s="17">
         <f>IFERROR(I6/$I$10,"-")</f>
-        <v>0.98888888888888893</v>
+        <v>0.99444444444444446</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -2360,15 +2376,15 @@
       </c>
       <c r="H8" s="27">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="16">
         <f>IFERROR(SUM(F8:H8),"-")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" s="17">
         <f>IFERROR(I8/$I$10,"-")</f>
-        <v>5.5555555555555558E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
@@ -2492,13 +2508,13 @@
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="21">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="C14" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>231</v>
+        <v>252</v>
       </c>
       <c r="E14" s="24" t="s">
         <v>4</v>
@@ -2506,44 +2522,44 @@
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="24" t="s">
-        <v>9</v>
+        <v>282</v>
       </c>
       <c r="I14" s="25"/>
       <c r="J14" s="25"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="21">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>212</v>
+        <v>125</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>252</v>
+        <v>283</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
       <c r="H15" s="24" t="s">
-        <v>282</v>
+        <v>9</v>
       </c>
       <c r="I15" s="25"/>
       <c r="J15" s="25"/>
     </row>
-    <row r="16" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="21">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>125</v>
+        <v>212</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>260</v>
+        <v>231</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" s="24"/>
       <c r="G16" s="24"/>
@@ -2555,13 +2571,13 @@
     </row>
     <row r="17" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B17" s="21">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C17" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E17" s="24" t="s">
         <v>5</v>
@@ -2576,13 +2592,13 @@
     </row>
     <row r="18" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B18" s="21">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>262</v>
+        <v>125</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E18" s="24" t="s">
         <v>5</v>
@@ -2595,18 +2611,18 @@
       <c r="I18" s="25"/>
       <c r="J18" s="25"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B19" s="21">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>139</v>
+        <v>262</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
@@ -2618,16 +2634,16 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="21">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>264</v>
+        <v>139</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
@@ -2637,18 +2653,18 @@
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
     </row>
-    <row r="21" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="21">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
@@ -2658,15 +2674,15 @@
       <c r="I21" s="25"/>
       <c r="J21" s="25"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B22" s="21">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E22" s="24" t="s">
         <v>3</v>
@@ -2681,16 +2697,16 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="21">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
@@ -2702,16 +2718,16 @@
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="21">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
@@ -2721,15 +2737,15 @@
       <c r="I24" s="25"/>
       <c r="J24" s="25"/>
     </row>
-    <row r="25" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="21">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>139</v>
+        <v>272</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E25" s="24" t="s">
         <v>3</v>
@@ -2742,15 +2758,15 @@
       <c r="I25" s="25"/>
       <c r="J25" s="25"/>
     </row>
-    <row r="26" spans="2:10" ht="54" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B26" s="21">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E26" s="24" t="s">
         <v>3</v>
@@ -2763,18 +2779,18 @@
       <c r="I26" s="25"/>
       <c r="J26" s="25"/>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" ht="54" x14ac:dyDescent="0.25">
       <c r="B27" s="21">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>276</v>
+        <v>162</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" s="24"/>
       <c r="G27" s="24"/>
@@ -2784,15 +2800,15 @@
       <c r="I27" s="25"/>
       <c r="J27" s="25"/>
     </row>
-    <row r="28" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="21">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C28" s="22" t="s">
         <v>276</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E28" s="24" t="s">
         <v>4</v>
@@ -2805,15 +2821,15 @@
       <c r="I28" s="25"/>
       <c r="J28" s="25"/>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B29" s="21">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>202</v>
+        <v>276</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E29" s="24" t="s">
         <v>4</v>
@@ -2826,15 +2842,15 @@
       <c r="I29" s="25"/>
       <c r="J29" s="25"/>
     </row>
-    <row r="30" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="21">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>139</v>
+        <v>202</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E30" s="24" t="s">
         <v>4</v>
@@ -2847,18 +2863,18 @@
       <c r="I30" s="25"/>
       <c r="J30" s="25"/>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B31" s="21">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>25</v>
+        <v>280</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" s="24"/>
       <c r="G31" s="24"/>
@@ -2870,16 +2886,16 @@
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E32" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F32" s="24"/>
       <c r="G32" s="24"/>
@@ -2891,13 +2907,13 @@
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E33" s="24" t="s">
         <v>5</v>
@@ -2912,16 +2928,16 @@
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="21">
+        <v>3</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34" s="24" t="s">
         <v>5</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>4</v>
       </c>
       <c r="F34" s="24"/>
       <c r="G34" s="24"/>
@@ -2933,16 +2949,16 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E35" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" s="24"/>
       <c r="G35" s="24"/>
@@ -2954,16 +2970,16 @@
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E36" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F36" s="24"/>
       <c r="G36" s="24"/>
@@ -2975,13 +2991,13 @@
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E37" s="24" t="s">
         <v>4</v>
@@ -2996,16 +3012,16 @@
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E38" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="24"/>
       <c r="G38" s="24"/>
@@ -3017,16 +3033,16 @@
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E39" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F39" s="24"/>
       <c r="G39" s="24"/>
@@ -3038,13 +3054,13 @@
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="21">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E40" s="24" t="s">
         <v>4</v>
@@ -3059,13 +3075,13 @@
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" s="21">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E41" s="24" t="s">
         <v>4</v>
@@ -3080,16 +3096,16 @@
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" s="21">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E42" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" s="24"/>
       <c r="G42" s="24"/>
@@ -3101,16 +3117,16 @@
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="21">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E43" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="24"/>
       <c r="G43" s="24"/>
@@ -3122,13 +3138,13 @@
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="21">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E44" s="24" t="s">
         <v>4</v>
@@ -3143,16 +3159,16 @@
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" s="21">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E45" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" s="24"/>
       <c r="G45" s="24"/>
@@ -3162,15 +3178,15 @@
       <c r="I45" s="25"/>
       <c r="J45" s="25"/>
     </row>
-    <row r="46" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="21">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E46" s="24" t="s">
         <v>5</v>
@@ -3183,15 +3199,15 @@
       <c r="I46" s="25"/>
       <c r="J46" s="25"/>
     </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B47" s="21">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E47" s="24" t="s">
         <v>5</v>
@@ -3206,16 +3222,16 @@
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="21">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E48" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F48" s="24"/>
       <c r="G48" s="24"/>
@@ -3225,15 +3241,15 @@
       <c r="I48" s="25"/>
       <c r="J48" s="25"/>
     </row>
-    <row r="49" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" s="21">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E49" s="24" t="s">
         <v>4</v>
@@ -3246,18 +3262,18 @@
       <c r="I49" s="25"/>
       <c r="J49" s="25"/>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B50" s="21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E50" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F50" s="24"/>
       <c r="G50" s="24"/>
@@ -3269,13 +3285,13 @@
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="21">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E51" s="24" t="s">
         <v>3</v>
@@ -3290,21 +3306,19 @@
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B52" s="21">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E52" s="24" t="s">
         <v>3</v>
       </c>
       <c r="F52" s="24"/>
-      <c r="G52" s="24" t="s">
-        <v>68</v>
-      </c>
+      <c r="G52" s="24"/>
       <c r="H52" s="24" t="s">
         <v>9</v>
       </c>
@@ -3313,19 +3327,21 @@
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" s="21">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C53" s="22" t="s">
         <v>66</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E53" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
+      <c r="G53" s="24" t="s">
+        <v>68</v>
+      </c>
       <c r="H53" s="24" t="s">
         <v>9</v>
       </c>
@@ -3334,16 +3350,16 @@
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="21">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E54" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F54" s="24"/>
       <c r="G54" s="24"/>
@@ -3355,16 +3371,16 @@
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55" s="21">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E55" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F55" s="24"/>
       <c r="G55" s="24"/>
@@ -3376,13 +3392,13 @@
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56" s="21">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E56" s="24" t="s">
         <v>5</v>
@@ -3397,16 +3413,16 @@
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="21">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E57" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F57" s="24"/>
       <c r="G57" s="24"/>
@@ -3418,16 +3434,16 @@
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B58" s="21">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E58" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F58" s="24"/>
       <c r="G58" s="24"/>
@@ -3439,16 +3455,16 @@
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="21">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E59" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F59" s="24"/>
       <c r="G59" s="24"/>
@@ -3460,16 +3476,16 @@
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60" s="21">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E60" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" s="24"/>
       <c r="G60" s="24"/>
@@ -3481,13 +3497,13 @@
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B61" s="21">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E61" s="24" t="s">
         <v>4</v>
@@ -3502,16 +3518,16 @@
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B62" s="21">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E62" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F62" s="24"/>
       <c r="G62" s="24"/>
@@ -3523,16 +3539,16 @@
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B63" s="21">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E63" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F63" s="24"/>
       <c r="G63" s="24"/>
@@ -3544,13 +3560,13 @@
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="21">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E64" s="24" t="s">
         <v>5</v>
@@ -3565,16 +3581,16 @@
     </row>
     <row r="65" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B65" s="21">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E65" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F65" s="24"/>
       <c r="G65" s="24"/>
@@ -3586,13 +3602,13 @@
     </row>
     <row r="66" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B66" s="21">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E66" s="24" t="s">
         <v>4</v>
@@ -3607,13 +3623,13 @@
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B67" s="21">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C67" s="22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E67" s="24" t="s">
         <v>4</v>
@@ -3628,16 +3644,16 @@
     </row>
     <row r="68" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B68" s="21">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C68" s="22" t="s">
         <v>95</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E68" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68" s="24"/>
       <c r="G68" s="24"/>
@@ -3649,16 +3665,16 @@
     </row>
     <row r="69" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B69" s="21">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C69" s="22" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E69" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F69" s="24"/>
       <c r="G69" s="24"/>
@@ -3668,18 +3684,18 @@
       <c r="I69" s="25"/>
       <c r="J69" s="25"/>
     </row>
-    <row r="70" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B70" s="21">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C70" s="22" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E70" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F70" s="24"/>
       <c r="G70" s="24"/>
@@ -3689,15 +3705,15 @@
       <c r="I70" s="25"/>
       <c r="J70" s="25"/>
     </row>
-    <row r="71" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B71" s="21">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E71" s="24" t="s">
         <v>3</v>
@@ -3710,18 +3726,18 @@
       <c r="I71" s="25"/>
       <c r="J71" s="25"/>
     </row>
-    <row r="72" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B72" s="21">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C72" s="22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E72" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F72" s="24"/>
       <c r="G72" s="24"/>
@@ -3731,15 +3747,15 @@
       <c r="I72" s="25"/>
       <c r="J72" s="25"/>
     </row>
-    <row r="73" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B73" s="21">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C73" s="22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E73" s="24" t="s">
         <v>5</v>
@@ -3754,13 +3770,13 @@
     </row>
     <row r="74" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B74" s="21">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C74" s="22" t="s">
         <v>105</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E74" s="24" t="s">
         <v>5</v>
@@ -3775,16 +3791,16 @@
     </row>
     <row r="75" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B75" s="21">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C75" s="22" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F75" s="24"/>
       <c r="G75" s="24"/>
@@ -3796,16 +3812,16 @@
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B76" s="21">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C76" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E76" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="24"/>
       <c r="G76" s="24"/>
@@ -3817,16 +3833,16 @@
     </row>
     <row r="77" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B77" s="21">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C77" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E77" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F77" s="24"/>
       <c r="G77" s="24"/>
@@ -3838,16 +3854,16 @@
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B78" s="21">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C78" s="22" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E78" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F78" s="24"/>
       <c r="G78" s="24"/>
@@ -3859,16 +3875,16 @@
     </row>
     <row r="79" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B79" s="21">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C79" s="22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E79" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F79" s="24"/>
       <c r="G79" s="24"/>
@@ -3880,16 +3896,16 @@
     </row>
     <row r="80" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B80" s="21">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C80" s="22" t="s">
         <v>116</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E80" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" s="24"/>
       <c r="G80" s="24"/>
@@ -3901,16 +3917,16 @@
     </row>
     <row r="81" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B81" s="21">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C81" s="22" t="s">
         <v>116</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E81" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" s="24"/>
       <c r="G81" s="24"/>
@@ -3920,18 +3936,18 @@
       <c r="I81" s="25"/>
       <c r="J81" s="25"/>
     </row>
-    <row r="82" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B82" s="21">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C82" s="22" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E82" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F82" s="24"/>
       <c r="G82" s="24"/>
@@ -3941,18 +3957,18 @@
       <c r="I82" s="25"/>
       <c r="J82" s="25"/>
     </row>
-    <row r="83" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B83" s="21">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C83" s="22" t="s">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="D83" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E83" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F83" s="24"/>
       <c r="G83" s="24"/>
@@ -3964,13 +3980,13 @@
     </row>
     <row r="84" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B84" s="21">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C84" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D84" s="23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E84" s="24" t="s">
         <v>3</v>
@@ -3985,13 +4001,13 @@
     </row>
     <row r="85" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B85" s="21">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C85" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D85" s="23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E85" s="24" t="s">
         <v>3</v>
@@ -4006,13 +4022,13 @@
     </row>
     <row r="86" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B86" s="21">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C86" s="22" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="D86" s="23" t="s">
-        <v>181</v>
+        <v>124</v>
       </c>
       <c r="E86" s="24" t="s">
         <v>3</v>
@@ -4027,16 +4043,16 @@
     </row>
     <row r="87" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B87" s="21">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C87" s="22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D87" s="23" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="E87" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F87" s="24"/>
       <c r="G87" s="24"/>
@@ -4048,16 +4064,16 @@
     </row>
     <row r="88" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B88" s="21">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C88" s="22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D88" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E88" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F88" s="24"/>
       <c r="G88" s="24"/>
@@ -4069,13 +4085,13 @@
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B89" s="21">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C89" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D89" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E89" s="24" t="s">
         <v>3</v>
@@ -4090,13 +4106,13 @@
     </row>
     <row r="90" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B90" s="21">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C90" s="22" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D90" s="23" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E90" s="24" t="s">
         <v>3</v>
@@ -4109,18 +4125,18 @@
       <c r="I90" s="25"/>
       <c r="J90" s="25"/>
     </row>
-    <row r="91" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B91" s="21">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C91" s="22" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="E91" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F91" s="24"/>
       <c r="G91" s="24"/>
@@ -4130,18 +4146,18 @@
       <c r="I91" s="25"/>
       <c r="J91" s="25"/>
     </row>
-    <row r="92" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B92" s="21">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C92" s="22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D92" s="23" t="s">
-        <v>134</v>
+        <v>170</v>
       </c>
       <c r="E92" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F92" s="24"/>
       <c r="G92" s="24"/>
@@ -4151,18 +4167,18 @@
       <c r="I92" s="25"/>
       <c r="J92" s="25"/>
     </row>
-    <row r="93" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B93" s="21">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C93" s="22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D93" s="23" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E93" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" s="24"/>
       <c r="G93" s="24"/>
@@ -4174,16 +4190,16 @@
     </row>
     <row r="94" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B94" s="21">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C94" s="22" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="D94" s="23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E94" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F94" s="24"/>
       <c r="G94" s="24"/>
@@ -4193,15 +4209,15 @@
       <c r="I94" s="25"/>
       <c r="J94" s="25"/>
     </row>
-    <row r="95" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B95" s="21">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C95" s="22" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="D95" s="23" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E95" s="24" t="s">
         <v>3</v>
@@ -4214,15 +4230,15 @@
       <c r="I95" s="25"/>
       <c r="J95" s="25"/>
     </row>
-    <row r="96" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B96" s="21">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C96" s="22" t="s">
-        <v>139</v>
+        <v>34</v>
       </c>
       <c r="D96" s="23" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E96" s="24" t="s">
         <v>3</v>
@@ -4237,13 +4253,13 @@
     </row>
     <row r="97" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B97" s="21">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C97" s="22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D97" s="23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E97" s="24" t="s">
         <v>3</v>
@@ -4256,18 +4272,18 @@
       <c r="I97" s="25"/>
       <c r="J97" s="25"/>
     </row>
-    <row r="98" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B98" s="21">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C98" s="22" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="D98" s="23" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E98" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" s="24"/>
       <c r="G98" s="24"/>
@@ -4277,18 +4293,18 @@
       <c r="I98" s="25"/>
       <c r="J98" s="25"/>
     </row>
-    <row r="99" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B99" s="21">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C99" s="22" t="s">
         <v>130</v>
       </c>
       <c r="D99" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F99" s="24"/>
       <c r="G99" s="24"/>
@@ -4298,18 +4314,18 @@
       <c r="I99" s="25"/>
       <c r="J99" s="25"/>
     </row>
-    <row r="100" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B100" s="21">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C100" s="22" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="D100" s="23" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E100" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F100" s="24"/>
       <c r="G100" s="24"/>
@@ -4321,16 +4337,16 @@
     </row>
     <row r="101" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B101" s="21">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C101" s="22" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="D101" s="23" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F101" s="24"/>
       <c r="G101" s="24"/>
@@ -4340,15 +4356,15 @@
       <c r="I101" s="25"/>
       <c r="J101" s="25"/>
     </row>
-    <row r="102" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B102" s="21">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C102" s="22" t="s">
         <v>110</v>
       </c>
       <c r="D102" s="23" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E102" s="24" t="s">
         <v>4</v>
@@ -4361,15 +4377,15 @@
       <c r="I102" s="25"/>
       <c r="J102" s="25"/>
     </row>
-    <row r="103" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B103" s="21">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C103" s="22" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="D103" s="23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E103" s="24" t="s">
         <v>4</v>
@@ -4382,18 +4398,18 @@
       <c r="I103" s="25"/>
       <c r="J103" s="25"/>
     </row>
-    <row r="104" spans="2:10" ht="121.5" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B104" s="21">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C104" s="22" t="s">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="D104" s="23" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E104" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F104" s="24"/>
       <c r="G104" s="24"/>
@@ -4403,15 +4419,15 @@
       <c r="I104" s="25"/>
       <c r="J104" s="25"/>
     </row>
-    <row r="105" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:10" ht="121.5" x14ac:dyDescent="0.25">
       <c r="B105" s="21">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C105" s="22" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D105" s="23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E105" s="24" t="s">
         <v>3</v>
@@ -4426,15 +4442,17 @@
     </row>
     <row r="106" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B106" s="21">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C106" s="22" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="D106" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="E106" s="24"/>
+        <v>153</v>
+      </c>
+      <c r="E106" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="F106" s="24"/>
       <c r="G106" s="24"/>
       <c r="H106" s="24" t="s">
@@ -4443,19 +4461,17 @@
       <c r="I106" s="25"/>
       <c r="J106" s="25"/>
     </row>
-    <row r="107" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B107" s="21">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C107" s="22" t="s">
         <v>130</v>
       </c>
       <c r="D107" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="E107" s="24" t="s">
-        <v>4</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="E107" s="24"/>
       <c r="F107" s="24"/>
       <c r="G107" s="24"/>
       <c r="H107" s="24" t="s">
@@ -4464,18 +4480,18 @@
       <c r="I107" s="25"/>
       <c r="J107" s="25"/>
     </row>
-    <row r="108" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B108" s="21">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C108" s="22" t="s">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="D108" s="23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E108" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F108" s="24"/>
       <c r="G108" s="24"/>
@@ -4487,16 +4503,16 @@
     </row>
     <row r="109" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B109" s="21">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C109" s="22" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D109" s="23" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E109" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F109" s="24"/>
       <c r="G109" s="24"/>
@@ -4506,18 +4522,18 @@
       <c r="I109" s="25"/>
       <c r="J109" s="25"/>
     </row>
-    <row r="110" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B110" s="21">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C110" s="22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D110" s="23" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E110" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F110" s="24"/>
       <c r="G110" s="24"/>
@@ -4527,18 +4543,18 @@
       <c r="I110" s="25"/>
       <c r="J110" s="25"/>
     </row>
-    <row r="111" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B111" s="21">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C111" s="22" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D111" s="23" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="E111" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F111" s="24"/>
       <c r="G111" s="24"/>
@@ -4548,18 +4564,18 @@
       <c r="I111" s="25"/>
       <c r="J111" s="25"/>
     </row>
-    <row r="112" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B112" s="21">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C112" s="22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D112" s="23" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E112" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F112" s="24"/>
       <c r="G112" s="24"/>
@@ -4571,16 +4587,16 @@
     </row>
     <row r="113" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B113" s="21">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C113" s="22" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D113" s="23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E113" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F113" s="24"/>
       <c r="G113" s="24"/>
@@ -4592,16 +4608,16 @@
     </row>
     <row r="114" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B114" s="21">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C114" s="22" t="s">
-        <v>125</v>
+        <v>165</v>
       </c>
       <c r="D114" s="23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E114" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F114" s="24"/>
       <c r="G114" s="24"/>
@@ -4611,18 +4627,18 @@
       <c r="I114" s="25"/>
       <c r="J114" s="25"/>
     </row>
-    <row r="115" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B115" s="21">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C115" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D115" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E115" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F115" s="24"/>
       <c r="G115" s="24"/>
@@ -4632,18 +4648,18 @@
       <c r="I115" s="25"/>
       <c r="J115" s="25"/>
     </row>
-    <row r="116" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B116" s="21">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C116" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D116" s="23" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E116" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F116" s="24"/>
       <c r="G116" s="24"/>
@@ -4653,18 +4669,18 @@
       <c r="I116" s="25"/>
       <c r="J116" s="25"/>
     </row>
-    <row r="117" spans="2:10" ht="81" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B117" s="21">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C117" s="22" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="D117" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E117" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F117" s="24"/>
       <c r="G117" s="24"/>
@@ -4674,15 +4690,15 @@
       <c r="I117" s="25"/>
       <c r="J117" s="25"/>
     </row>
-    <row r="118" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:10" ht="81" x14ac:dyDescent="0.25">
       <c r="B118" s="21">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C118" s="22" t="s">
         <v>95</v>
       </c>
       <c r="D118" s="23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E118" s="24" t="s">
         <v>4</v>
@@ -4695,18 +4711,18 @@
       <c r="I118" s="25"/>
       <c r="J118" s="25"/>
     </row>
-    <row r="119" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B119" s="21">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C119" s="22" t="s">
-        <v>174</v>
+        <v>95</v>
       </c>
       <c r="D119" s="23" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E119" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F119" s="24"/>
       <c r="G119" s="24"/>
@@ -4718,13 +4734,13 @@
     </row>
     <row r="120" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B120" s="21">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C120" s="22" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="D120" s="23" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E120" s="24" t="s">
         <v>3</v>
@@ -4739,16 +4755,16 @@
     </row>
     <row r="121" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B121" s="21">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C121" s="22" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D121" s="23" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E121" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F121" s="24"/>
       <c r="G121" s="24"/>
@@ -4758,18 +4774,18 @@
       <c r="I121" s="25"/>
       <c r="J121" s="25"/>
     </row>
-    <row r="122" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B122" s="21">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C122" s="22" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="D122" s="23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E122" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F122" s="24"/>
       <c r="G122" s="24"/>
@@ -4779,18 +4795,18 @@
       <c r="I122" s="25"/>
       <c r="J122" s="25"/>
     </row>
-    <row r="123" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B123" s="21">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C123" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D123" s="23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E123" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F123" s="24"/>
       <c r="G123" s="24"/>
@@ -4802,16 +4818,16 @@
     </row>
     <row r="124" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B124" s="21">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C124" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D124" s="23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E124" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F124" s="24"/>
       <c r="G124" s="24"/>
@@ -4823,13 +4839,13 @@
     </row>
     <row r="125" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B125" s="21">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C125" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D125" s="23" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E125" s="24" t="s">
         <v>3</v>
@@ -4844,16 +4860,16 @@
     </row>
     <row r="126" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B126" s="21">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C126" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D126" s="23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E126" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F126" s="24"/>
       <c r="G126" s="24"/>
@@ -4863,18 +4879,18 @@
       <c r="I126" s="25"/>
       <c r="J126" s="25"/>
     </row>
-    <row r="127" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B127" s="21">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C127" s="22" t="s">
-        <v>162</v>
+        <v>125</v>
       </c>
       <c r="D127" s="23" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E127" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F127" s="24"/>
       <c r="G127" s="24"/>
@@ -4884,18 +4900,18 @@
       <c r="I127" s="25"/>
       <c r="J127" s="25"/>
     </row>
-    <row r="128" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B128" s="21">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C128" s="22" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="D128" s="23" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E128" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F128" s="24"/>
       <c r="G128" s="24"/>
@@ -4907,13 +4923,13 @@
     </row>
     <row r="129" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B129" s="21">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C129" s="22" t="s">
-        <v>120</v>
+        <v>185</v>
       </c>
       <c r="D129" s="23" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E129" s="24" t="s">
         <v>5</v>
@@ -4926,18 +4942,18 @@
       <c r="I129" s="25"/>
       <c r="J129" s="25"/>
     </row>
-    <row r="130" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B130" s="21">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C130" s="22" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D130" s="23" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E130" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F130" s="24"/>
       <c r="G130" s="24"/>
@@ -4947,18 +4963,18 @@
       <c r="I130" s="25"/>
       <c r="J130" s="25"/>
     </row>
-    <row r="131" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B131" s="21">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C131" s="22" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="D131" s="23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E131" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F131" s="24"/>
       <c r="G131" s="24"/>
@@ -4970,16 +4986,16 @@
     </row>
     <row r="132" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B132" s="21">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C132" s="22" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D132" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E132" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F132" s="24"/>
       <c r="G132" s="24"/>
@@ -4991,16 +5007,16 @@
     </row>
     <row r="133" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B133" s="21">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C133" s="22" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D133" s="23" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E133" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F133" s="24"/>
       <c r="G133" s="24"/>
@@ -5012,16 +5028,16 @@
     </row>
     <row r="134" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B134" s="21">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C134" s="22" t="s">
         <v>125</v>
       </c>
       <c r="D134" s="23" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E134" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F134" s="24"/>
       <c r="G134" s="24"/>
@@ -5031,18 +5047,18 @@
       <c r="I134" s="25"/>
       <c r="J134" s="25"/>
     </row>
-    <row r="135" spans="2:10" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B135" s="21">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C135" s="22" t="s">
-        <v>193</v>
+        <v>125</v>
       </c>
       <c r="D135" s="23" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E135" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F135" s="24"/>
       <c r="G135" s="24"/>
@@ -5052,18 +5068,18 @@
       <c r="I135" s="25"/>
       <c r="J135" s="25"/>
     </row>
-    <row r="136" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:10" ht="67.5" x14ac:dyDescent="0.25">
       <c r="B136" s="21">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C136" s="22" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="D136" s="23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E136" s="24" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F136" s="24"/>
       <c r="G136" s="24"/>
@@ -5075,16 +5091,16 @@
     </row>
     <row r="137" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B137" s="21">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C137" s="22" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="D137" s="23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E137" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F137" s="24"/>
       <c r="G137" s="24"/>
@@ -5096,13 +5112,13 @@
     </row>
     <row r="138" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B138" s="21">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C138" s="22" t="s">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="D138" s="23" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E138" s="24" t="s">
         <v>5</v>
@@ -5117,16 +5133,16 @@
     </row>
     <row r="139" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B139" s="21">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C139" s="22" t="s">
         <v>197</v>
       </c>
       <c r="D139" s="23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E139" s="24" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F139" s="24"/>
       <c r="G139" s="24"/>
@@ -5138,13 +5154,13 @@
     </row>
     <row r="140" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B140" s="21">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C140" s="22" t="s">
         <v>197</v>
       </c>
       <c r="D140" s="23" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E140" s="24" t="s">
         <v>3</v>
@@ -5159,13 +5175,13 @@
     </row>
     <row r="141" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B141" s="21">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C141" s="22" t="s">
-        <v>139</v>
+        <v>197</v>
       </c>
       <c r="D141" s="23" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E141" s="24" t="s">
         <v>3</v>
@@ -5178,15 +5194,15 @@
       <c r="I141" s="25"/>
       <c r="J141" s="25"/>
     </row>
-    <row r="142" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B142" s="21">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C142" s="22" t="s">
-        <v>202</v>
+        <v>139</v>
       </c>
       <c r="D142" s="23" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E142" s="24" t="s">
         <v>3</v>
@@ -5201,16 +5217,16 @@
     </row>
     <row r="143" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B143" s="21">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C143" s="22" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="D143" s="23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E143" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F143" s="24"/>
       <c r="G143" s="24"/>
@@ -5220,18 +5236,18 @@
       <c r="I143" s="25"/>
       <c r="J143" s="25"/>
     </row>
-    <row r="144" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B144" s="21">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C144" s="22" t="s">
-        <v>130</v>
+        <v>163</v>
       </c>
       <c r="D144" s="23" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E144" s="24" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F144" s="24"/>
       <c r="G144" s="24"/>
@@ -5241,15 +5257,15 @@
       <c r="I144" s="25"/>
       <c r="J144" s="25"/>
     </row>
-    <row r="145" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B145" s="21">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C145" s="22" t="s">
-        <v>206</v>
+        <v>130</v>
       </c>
       <c r="D145" s="23" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E145" s="24" t="s">
         <v>3</v>
@@ -5262,15 +5278,15 @@
       <c r="I145" s="25"/>
       <c r="J145" s="25"/>
     </row>
-    <row r="146" spans="2:10" ht="27" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B146" s="21">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C146" s="22" t="s">
-        <v>156</v>
+        <v>206</v>
       </c>
       <c r="D146" s="23" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E146" s="24" t="s">
         <v>3</v>
@@ -5283,15 +5299,15 @@
       <c r="I146" s="25"/>
       <c r="J146" s="25"/>
     </row>
-    <row r="147" spans="2:10" ht="108" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B147" s="21">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C147" s="22" t="s">
-        <v>116</v>
+        <v>156</v>
       </c>
       <c r="D147" s="23" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E147" s="24" t="s">
         <v>3</v>
@@ -5304,15 +5320,15 @@
       <c r="I147" s="25"/>
       <c r="J147" s="25"/>
     </row>
-    <row r="148" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:10" ht="108" x14ac:dyDescent="0.25">
       <c r="B148" s="21">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C148" s="22" t="s">
-        <v>210</v>
+        <v>116</v>
       </c>
       <c r="D148" s="23" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E148" s="24" t="s">
         <v>3</v>
@@ -5327,16 +5343,16 @@
     </row>
     <row r="149" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B149" s="21">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C149" s="22" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D149" s="23" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E149" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F149" s="24"/>
       <c r="G149" s="24"/>
@@ -5348,13 +5364,13 @@
     </row>
     <row r="150" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B150" s="21">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C150" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D150" s="23" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E150" s="24" t="s">
         <v>4</v>
@@ -5369,13 +5385,13 @@
     </row>
     <row r="151" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B151" s="21">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C151" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D151" s="23" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E151" s="24" t="s">
         <v>4</v>
@@ -5390,13 +5406,13 @@
     </row>
     <row r="152" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B152" s="21">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C152" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D152" s="23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E152" s="24" t="s">
         <v>4</v>
@@ -5411,13 +5427,13 @@
     </row>
     <row r="153" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B153" s="21">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C153" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D153" s="23" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E153" s="24" t="s">
         <v>4</v>
@@ -5432,13 +5448,13 @@
     </row>
     <row r="154" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B154" s="21">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C154" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D154" s="23" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E154" s="24" t="s">
         <v>4</v>
@@ -5453,13 +5469,13 @@
     </row>
     <row r="155" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B155" s="21">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C155" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D155" s="23" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E155" s="24" t="s">
         <v>4</v>
@@ -5474,13 +5490,13 @@
     </row>
     <row r="156" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B156" s="21">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C156" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D156" s="23" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E156" s="24" t="s">
         <v>4</v>
@@ -5495,13 +5511,13 @@
     </row>
     <row r="157" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B157" s="21">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C157" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D157" s="23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E157" s="24" t="s">
         <v>4</v>
@@ -5516,13 +5532,13 @@
     </row>
     <row r="158" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B158" s="21">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C158" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D158" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E158" s="24" t="s">
         <v>4</v>
@@ -5537,13 +5553,13 @@
     </row>
     <row r="159" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B159" s="21">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C159" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D159" s="23" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E159" s="24" t="s">
         <v>4</v>
@@ -5558,13 +5574,13 @@
     </row>
     <row r="160" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B160" s="21">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C160" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D160" s="23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E160" s="24" t="s">
         <v>4</v>
@@ -5579,13 +5595,13 @@
     </row>
     <row r="161" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B161" s="21">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C161" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D161" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E161" s="24" t="s">
         <v>4</v>
@@ -5600,13 +5616,13 @@
     </row>
     <row r="162" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B162" s="21">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C162" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D162" s="23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E162" s="24" t="s">
         <v>4</v>
@@ -5621,13 +5637,13 @@
     </row>
     <row r="163" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B163" s="21">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C163" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D163" s="23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E163" s="24" t="s">
         <v>4</v>
@@ -5642,13 +5658,13 @@
     </row>
     <row r="164" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B164" s="21">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C164" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D164" s="23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E164" s="24" t="s">
         <v>4</v>
@@ -5663,13 +5679,13 @@
     </row>
     <row r="165" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B165" s="21">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C165" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D165" s="23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E165" s="24" t="s">
         <v>4</v>
@@ -5684,13 +5700,13 @@
     </row>
     <row r="166" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B166" s="21">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C166" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D166" s="23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E166" s="24" t="s">
         <v>4</v>
@@ -5705,13 +5721,13 @@
     </row>
     <row r="167" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B167" s="21">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C167" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D167" s="23" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E167" s="24" t="s">
         <v>4</v>
@@ -5726,13 +5742,13 @@
     </row>
     <row r="168" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B168" s="21">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C168" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D168" s="23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E168" s="24" t="s">
         <v>4</v>
@@ -5747,13 +5763,13 @@
     </row>
     <row r="169" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B169" s="21">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C169" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D169" s="23" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E169" s="24" t="s">
         <v>4</v>
@@ -5768,13 +5784,13 @@
     </row>
     <row r="170" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B170" s="21">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C170" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D170" s="23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E170" s="24" t="s">
         <v>4</v>
@@ -5789,13 +5805,13 @@
     </row>
     <row r="171" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B171" s="21">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C171" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D171" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E171" s="24" t="s">
         <v>4</v>
@@ -5810,13 +5826,13 @@
     </row>
     <row r="172" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B172" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C172" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D172" s="23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E172" s="24" t="s">
         <v>4</v>
@@ -5831,13 +5847,13 @@
     </row>
     <row r="173" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B173" s="21">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C173" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D173" s="23" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E173" s="24" t="s">
         <v>4</v>
@@ -5852,13 +5868,13 @@
     </row>
     <row r="174" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B174" s="21">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C174" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D174" s="23" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E174" s="24" t="s">
         <v>4</v>
@@ -5873,13 +5889,13 @@
     </row>
     <row r="175" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B175" s="21">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C175" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D175" s="23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E175" s="24" t="s">
         <v>4</v>
@@ -5894,13 +5910,13 @@
     </row>
     <row r="176" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B176" s="21">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C176" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E176" s="24" t="s">
         <v>4</v>
@@ -5915,13 +5931,13 @@
     </row>
     <row r="177" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B177" s="21">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C177" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D177" s="23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E177" s="24" t="s">
         <v>4</v>
@@ -5936,13 +5952,13 @@
     </row>
     <row r="178" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B178" s="21">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C178" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D178" s="23" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E178" s="24" t="s">
         <v>4</v>
@@ -5957,13 +5973,13 @@
     </row>
     <row r="179" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B179" s="21">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C179" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D179" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E179" s="24" t="s">
         <v>4</v>
@@ -5978,13 +5994,13 @@
     </row>
     <row r="180" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B180" s="21">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C180" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D180" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E180" s="24" t="s">
         <v>4</v>
@@ -5999,13 +6015,13 @@
     </row>
     <row r="181" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B181" s="21">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C181" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D181" s="23" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E181" s="24" t="s">
         <v>4</v>
@@ -6020,13 +6036,13 @@
     </row>
     <row r="182" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B182" s="21">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C182" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D182" s="23" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E182" s="24" t="s">
         <v>4</v>
@@ -6041,13 +6057,13 @@
     </row>
     <row r="183" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B183" s="21">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C183" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D183" s="23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E183" s="24" t="s">
         <v>4</v>
@@ -6062,13 +6078,13 @@
     </row>
     <row r="184" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B184" s="21">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C184" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D184" s="23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E184" s="24" t="s">
         <v>4</v>
@@ -6083,13 +6099,13 @@
     </row>
     <row r="185" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B185" s="21">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C185" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D185" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E185" s="24" t="s">
         <v>4</v>
@@ -6104,13 +6120,13 @@
     </row>
     <row r="186" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B186" s="21">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C186" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D186" s="23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E186" s="24" t="s">
         <v>4</v>
@@ -6125,13 +6141,13 @@
     </row>
     <row r="187" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B187" s="21">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C187" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D187" s="23" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E187" s="24" t="s">
         <v>4</v>
@@ -6146,13 +6162,13 @@
     </row>
     <row r="188" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B188" s="21">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C188" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D188" s="23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E188" s="24" t="s">
         <v>4</v>
@@ -6167,13 +6183,13 @@
     </row>
     <row r="189" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B189" s="21">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C189" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D189" s="23" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E189" s="24" t="s">
         <v>4</v>
@@ -6188,13 +6204,13 @@
     </row>
     <row r="190" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B190" s="21">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C190" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D190" s="23" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E190" s="24" t="s">
         <v>4</v>
@@ -6209,13 +6225,13 @@
     </row>
     <row r="191" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B191" s="21">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C191" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D191" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E191" s="24" t="s">
         <v>4</v>
@@ -6230,13 +6246,13 @@
     </row>
     <row r="192" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B192" s="21">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C192" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D192" s="23" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E192" s="24" t="s">
         <v>4</v>
@@ -6251,13 +6267,13 @@
     </row>
     <row r="193" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B193" s="21">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C193" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D193" s="23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E193" s="24" t="s">
         <v>4</v>
@@ -6272,21 +6288,21 @@
     </row>
     <row r="194" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B194" s="21">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C194" s="22" t="s">
-        <v>125</v>
+        <v>212</v>
       </c>
       <c r="D194" s="23" t="s">
-        <v>283</v>
+        <v>259</v>
       </c>
       <c r="E194" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F194" s="24"/>
       <c r="G194" s="24"/>
       <c r="H194" s="24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I194" s="25"/>
       <c r="J194" s="25"/>
@@ -6893,13 +6909,13 @@
     <mergeCell ref="B8:B9"/>
   </mergeCells>
   <conditionalFormatting sqref="B13:J247">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$H13="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$H13="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$H13="Retest"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Internationalize public marketing pages and admin interface with translation function calls and locale support
Replace hardcoded English text with t() translation function calls across 404.php, about.php, admin-practices.php, and accept-baa.php, add getHtmlLang() calls to <html lang> attributes, add renderLanguageSelector() to navigation, replace inline text with translation keys for SEO meta tags/navigation/content/footer/admin stats/table headers/buttons/modals/API responses, add default_locale column to practice creation, pass practiceId to sendWelcomeEmail for locale-aware emails, add
</commit_message>
<xml_diff>
--- a/documentation/Issue Tracker.xlsx
+++ b/documentation/Issue Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAMP\htdocs\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAMP\htdocs\DentaTrak\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCB103E-706F-437F-9246-304D43ED5E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F94694-3C51-4090-840C-C7330D143225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B30AA0F8-B590-4D13-9530-2CA817625601}"/>
+    <workbookView xWindow="2985" yWindow="3105" windowWidth="21600" windowHeight="11295" xr2:uid="{B30AA0F8-B590-4D13-9530-2CA817625601}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="308">
   <si>
     <t>ISSUE TRACKER</t>
   </si>
@@ -895,6 +895,78 @@
   </si>
   <si>
     <t>Keeps the login with email section expanded and it's driving me nuts</t>
+  </si>
+  <si>
+    <t>Lab Insights</t>
+  </si>
+  <si>
+    <t>The tooltips in the header of lab performance are all caps and have things like started_at. Also need to verify that its calculating those correctly</t>
+  </si>
+  <si>
+    <t>Resources</t>
+  </si>
+  <si>
+    <t>Need to update resources page for better catorization</t>
+  </si>
+  <si>
+    <t>Add tracking spreadsheet to resources page</t>
+  </si>
+  <si>
+    <t>Update site for better mobile experience</t>
+  </si>
+  <si>
+    <t>Accessability</t>
+  </si>
+  <si>
+    <t>Make sure site is accessibile and ADA compliant</t>
+  </si>
+  <si>
+    <t>Internationalization</t>
+  </si>
+  <si>
+    <t>Add spanish</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>Add notifications (email, app, text)</t>
+  </si>
+  <si>
+    <t>Secure Chat</t>
+  </si>
+  <si>
+    <t>Add secure chat</t>
+  </si>
+  <si>
+    <t>Update user guide</t>
+  </si>
+  <si>
+    <t>Translate user guide to spanish</t>
+  </si>
+  <si>
+    <t>Insights</t>
+  </si>
+  <si>
+    <t>Have a combined insights tab with sub tabs for practice and lab?</t>
+  </si>
+  <si>
+    <t>Landing Page</t>
+  </si>
+  <si>
+    <t>Swap Pricing and Resources in menu</t>
+  </si>
+  <si>
+    <t>Add HIPAA info</t>
+  </si>
+  <si>
+    <t>Make copy more compelling</t>
+  </si>
+  <si>
+    <t>Add Clear button to the filters</t>
+  </si>
+  <si>
+    <t>Add tagging and filters by tag</t>
   </si>
 </sst>
 </file>
@@ -1279,31 +1351,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill>
@@ -1557,6 +1605,14 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <strike val="0"/>
@@ -1661,9 +1717,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="3" xr9:uid="{9287C67C-ECEA-45B3-8051-FC9FD9595AF7}">
-      <tableStyleElement type="wholeTable" dxfId="19"/>
-      <tableStyleElement type="firstRowStripe" dxfId="18"/>
-      <tableStyleElement type="secondRowStripe" dxfId="17"/>
+      <tableStyleElement type="wholeTable" dxfId="17"/>
+      <tableStyleElement type="firstRowStripe" dxfId="16"/>
+      <tableStyleElement type="secondRowStripe" dxfId="15"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1886,21 +1942,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}" name="TblMain" displayName="TblMain" ref="B13:J247" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="B13:J247" xr:uid="{7B58E07B-F9D0-41A5-AACF-5EAC85B8FC69}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B14:J247">
-    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="1"/>
+    <sortCondition sortBy="cellColor" ref="H13:H247" dxfId="12"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{C0EEC035-1A27-4C90-A172-7DFF5AB6F3C5}" name="#" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{CABC7F69-5311-4199-9383-8E2C3735E509}" name="ISSUE" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{6668E032-1895-4222-969B-7146FCA03F81}" name="DESCRIPTION" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{393780AC-67D6-42F6-8249-8924FB9342DC}" name="PRIORITY" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A5E66358-FEA1-4BCC-9899-00325DFBD8D8}" name="DEPARTMENT" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{E4346B87-DD68-4C69-871D-5F271B4A7AFF}" name="INITIATOR" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{E2C1F364-38D8-4098-92EB-5938C5417D7A}" name="STATUS" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{D4F26330-CA7E-44AB-A17C-68FA53720DD9}" name="OPENED ON" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{D3740E9D-E72E-4928-B430-F83B6FC283A9}" name="CLOSED ON" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2326,7 +2382,7 @@
       </c>
       <c r="J6" s="17">
         <f>IFERROR(I6/$I$10,"-")</f>
-        <v>0.99444444444444446</v>
+        <v>0.91326530612244894</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -2340,23 +2396,23 @@
       </c>
       <c r="F7" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H7" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="16">
         <f>IFERROR(SUM(F7:H7),"-")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J7" s="17">
         <f>IFERROR(I7/$I$10,"-")</f>
-        <v>0</v>
+        <v>3.5714285714285712E-2</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -2372,19 +2428,19 @@
       </c>
       <c r="G8" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H8" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8" s="16">
         <f>IFERROR(SUM(F8:H8),"-")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J8" s="17">
         <f>IFERROR(I8/$I$10,"-")</f>
-        <v>0</v>
+        <v>4.5918367346938778E-2</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
@@ -2412,7 +2468,7 @@
       </c>
       <c r="J9" s="17">
         <f>IFERROR(I9/$I$10,"-")</f>
-        <v>5.5555555555555558E-3</v>
+        <v>5.1020408163265302E-3</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
@@ -2426,19 +2482,19 @@
       </c>
       <c r="F10" s="16">
         <f>IFERROR(SUM(F6:F9),"-")</f>
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G10" s="16">
         <f>IFERROR(SUM(G6:G9),"-")</f>
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H10" s="16">
         <f>IFERROR(SUM(H6:H9),"-")</f>
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I10" s="16">
         <f>IFERROR(SUM(F10:H10),"-")</f>
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="J10" s="18"/>
     </row>
@@ -2453,15 +2509,15 @@
       </c>
       <c r="F11" s="17">
         <f>IFERROR(F10/$I$10,"-")</f>
-        <v>0.28888888888888886</v>
+        <v>0.28061224489795916</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" ref="G11:H11" si="1">IFERROR(G10/$I$10,"-")</f>
-        <v>0.51666666666666672</v>
+        <v>0.52551020408163263</v>
       </c>
       <c r="H11" s="17">
         <f t="shared" si="1"/>
-        <v>0.19444444444444445</v>
+        <v>0.19387755102040816</v>
       </c>
       <c r="I11" s="18"/>
       <c r="J11" s="19"/>
@@ -6307,179 +6363,339 @@
       <c r="I194" s="25"/>
       <c r="J194" s="25"/>
     </row>
-    <row r="195" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B195" s="21"/>
-      <c r="C195" s="22"/>
-      <c r="D195" s="23"/>
-      <c r="E195" s="24"/>
+    <row r="195" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="B195" s="21">
+        <v>179</v>
+      </c>
+      <c r="C195" s="22" t="s">
+        <v>284</v>
+      </c>
+      <c r="D195" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="E195" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F195" s="24"/>
       <c r="G195" s="24"/>
-      <c r="H195" s="24"/>
+      <c r="H195" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I195" s="25"/>
       <c r="J195" s="25"/>
     </row>
     <row r="196" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B196" s="21"/>
-      <c r="C196" s="22"/>
-      <c r="D196" s="23"/>
-      <c r="E196" s="24"/>
+      <c r="B196" s="21">
+        <v>180</v>
+      </c>
+      <c r="C196" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="D196" s="23" t="s">
+        <v>287</v>
+      </c>
+      <c r="E196" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F196" s="24"/>
       <c r="G196" s="24"/>
-      <c r="H196" s="24"/>
+      <c r="H196" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I196" s="25"/>
       <c r="J196" s="25"/>
     </row>
     <row r="197" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B197" s="21"/>
-      <c r="C197" s="22"/>
-      <c r="D197" s="23"/>
-      <c r="E197" s="24"/>
+      <c r="B197" s="21">
+        <v>181</v>
+      </c>
+      <c r="C197" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="D197" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="E197" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F197" s="24"/>
       <c r="G197" s="24"/>
-      <c r="H197" s="24"/>
+      <c r="H197" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I197" s="25"/>
       <c r="J197" s="25"/>
     </row>
     <row r="198" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B198" s="21"/>
-      <c r="C198" s="22"/>
-      <c r="D198" s="23"/>
-      <c r="E198" s="24"/>
+      <c r="B198" s="21">
+        <v>182</v>
+      </c>
+      <c r="C198" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="D198" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="E198" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F198" s="24"/>
       <c r="G198" s="24"/>
-      <c r="H198" s="24"/>
+      <c r="H198" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I198" s="25"/>
       <c r="J198" s="25"/>
     </row>
     <row r="199" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B199" s="21"/>
-      <c r="C199" s="22"/>
-      <c r="D199" s="23"/>
-      <c r="E199" s="24"/>
+      <c r="B199" s="21">
+        <v>183</v>
+      </c>
+      <c r="C199" s="22" t="s">
+        <v>290</v>
+      </c>
+      <c r="D199" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="E199" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F199" s="24"/>
       <c r="G199" s="24"/>
-      <c r="H199" s="24"/>
+      <c r="H199" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I199" s="25"/>
       <c r="J199" s="25"/>
     </row>
     <row r="200" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B200" s="21"/>
-      <c r="C200" s="22"/>
-      <c r="D200" s="23"/>
-      <c r="E200" s="24"/>
+      <c r="B200" s="21">
+        <v>184</v>
+      </c>
+      <c r="C200" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="D200" s="23" t="s">
+        <v>293</v>
+      </c>
+      <c r="E200" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F200" s="24"/>
       <c r="G200" s="24"/>
-      <c r="H200" s="24"/>
+      <c r="H200" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I200" s="25"/>
       <c r="J200" s="25"/>
     </row>
     <row r="201" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B201" s="21"/>
-      <c r="C201" s="22"/>
-      <c r="D201" s="23"/>
-      <c r="E201" s="24"/>
+      <c r="B201" s="21">
+        <v>185</v>
+      </c>
+      <c r="C201" s="22" t="s">
+        <v>294</v>
+      </c>
+      <c r="D201" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="E201" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F201" s="24"/>
       <c r="G201" s="24"/>
-      <c r="H201" s="24"/>
+      <c r="H201" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I201" s="25"/>
       <c r="J201" s="25"/>
     </row>
     <row r="202" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B202" s="21"/>
-      <c r="C202" s="22"/>
-      <c r="D202" s="23"/>
-      <c r="E202" s="24"/>
+      <c r="B202" s="21">
+        <v>186</v>
+      </c>
+      <c r="C202" s="22" t="s">
+        <v>296</v>
+      </c>
+      <c r="D202" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="E202" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F202" s="24"/>
       <c r="G202" s="24"/>
-      <c r="H202" s="24"/>
+      <c r="H202" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I202" s="25"/>
       <c r="J202" s="25"/>
     </row>
     <row r="203" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B203" s="21"/>
-      <c r="C203" s="22"/>
-      <c r="D203" s="23"/>
-      <c r="E203" s="24"/>
+      <c r="B203" s="21">
+        <v>187</v>
+      </c>
+      <c r="C203" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="D203" s="23" t="s">
+        <v>298</v>
+      </c>
+      <c r="E203" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F203" s="24"/>
       <c r="G203" s="24"/>
-      <c r="H203" s="24"/>
+      <c r="H203" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I203" s="25"/>
       <c r="J203" s="25"/>
     </row>
     <row r="204" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B204" s="21"/>
-      <c r="C204" s="22"/>
-      <c r="D204" s="23"/>
-      <c r="E204" s="24"/>
+      <c r="B204" s="21">
+        <v>188</v>
+      </c>
+      <c r="C204" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="D204" s="23" t="s">
+        <v>299</v>
+      </c>
+      <c r="E204" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F204" s="24"/>
       <c r="G204" s="24"/>
-      <c r="H204" s="24"/>
+      <c r="H204" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I204" s="25"/>
       <c r="J204" s="25"/>
     </row>
     <row r="205" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B205" s="21"/>
-      <c r="C205" s="22"/>
-      <c r="D205" s="23"/>
-      <c r="E205" s="24"/>
+      <c r="B205" s="21">
+        <v>189</v>
+      </c>
+      <c r="C205" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="D205" s="23" t="s">
+        <v>301</v>
+      </c>
+      <c r="E205" s="24" t="s">
+        <v>5</v>
+      </c>
       <c r="F205" s="24"/>
       <c r="G205" s="24"/>
-      <c r="H205" s="24"/>
+      <c r="H205" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I205" s="25"/>
       <c r="J205" s="25"/>
     </row>
     <row r="206" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B206" s="21"/>
-      <c r="C206" s="22"/>
-      <c r="D206" s="23"/>
-      <c r="E206" s="24"/>
+      <c r="B206" s="21">
+        <v>190</v>
+      </c>
+      <c r="C206" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="D206" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="E206" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="F206" s="24"/>
       <c r="G206" s="24"/>
-      <c r="H206" s="24"/>
+      <c r="H206" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I206" s="25"/>
       <c r="J206" s="25"/>
     </row>
     <row r="207" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B207" s="21"/>
-      <c r="C207" s="22"/>
-      <c r="D207" s="23"/>
-      <c r="E207" s="24"/>
+      <c r="B207" s="21">
+        <v>191</v>
+      </c>
+      <c r="C207" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D207" s="23" t="s">
+        <v>304</v>
+      </c>
+      <c r="E207" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="F207" s="24"/>
       <c r="G207" s="24"/>
-      <c r="H207" s="24"/>
+      <c r="H207" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I207" s="25"/>
       <c r="J207" s="25"/>
     </row>
     <row r="208" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B208" s="21"/>
-      <c r="C208" s="22"/>
-      <c r="D208" s="23"/>
-      <c r="E208" s="24"/>
+      <c r="B208" s="21">
+        <v>192</v>
+      </c>
+      <c r="C208" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="D208" s="23" t="s">
+        <v>305</v>
+      </c>
+      <c r="E208" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="F208" s="24"/>
       <c r="G208" s="24"/>
-      <c r="H208" s="24"/>
+      <c r="H208" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I208" s="25"/>
       <c r="J208" s="25"/>
     </row>
     <row r="209" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B209" s="21"/>
-      <c r="C209" s="22"/>
-      <c r="D209" s="23"/>
-      <c r="E209" s="24"/>
+      <c r="B209" s="21">
+        <v>193</v>
+      </c>
+      <c r="C209" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="D209" s="23" t="s">
+        <v>306</v>
+      </c>
+      <c r="E209" s="24" t="s">
+        <v>5</v>
+      </c>
       <c r="F209" s="24"/>
       <c r="G209" s="24"/>
-      <c r="H209" s="24"/>
+      <c r="H209" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I209" s="25"/>
       <c r="J209" s="25"/>
     </row>
     <row r="210" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B210" s="21"/>
-      <c r="C210" s="22"/>
-      <c r="D210" s="23"/>
-      <c r="E210" s="24"/>
+      <c r="B210" s="21">
+        <v>194</v>
+      </c>
+      <c r="C210" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D210" s="23" t="s">
+        <v>307</v>
+      </c>
+      <c r="E210" s="24" t="s">
+        <v>5</v>
+      </c>
       <c r="F210" s="24"/>
       <c r="G210" s="24"/>
-      <c r="H210" s="24"/>
+      <c r="H210" s="24" t="s">
+        <v>12</v>
+      </c>
       <c r="I210" s="25"/>
       <c r="J210" s="25"/>
     </row>
@@ -6909,13 +7125,13 @@
     <mergeCell ref="B8:B9"/>
   </mergeCells>
   <conditionalFormatting sqref="B13:J247">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$H13="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$H13="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$H13="Retest"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Add internationalization to admin practices page, compact UI styling, HIPAA security page routing, and fix lab insights turnaround/multi-lab calculations
Replace hardcoded English text with t() translation calls throughout admin-practices.php (title/tabs/status/loading/print/users/cases), add getHtmlLang() to <html lang> attribute, add 137 lines of compact UI CSS overrides for reduced padding/font-sizes across headers/stats/tables/panels/badges/tabs, add trial urgency styling classes (trial-urgent/
</commit_message>
<xml_diff>
--- a/documentation/Issue Tracker.xlsx
+++ b/documentation/Issue Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAMP\htdocs\DentaTrak\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F94694-3C51-4090-840C-C7330D143225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8026FB04-A972-4058-BB5F-AC90B95BC33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2985" yWindow="3105" windowWidth="21600" windowHeight="11295" xr2:uid="{B30AA0F8-B590-4D13-9530-2CA817625601}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="309">
   <si>
     <t>ISSUE TRACKER</t>
   </si>
@@ -967,6 +967,9 @@
   </si>
   <si>
     <t>Add tagging and filters by tag</t>
+  </si>
+  <si>
+    <t>Update DevTools and Practice Administration</t>
   </si>
 </sst>
 </file>
@@ -2366,23 +2369,23 @@
       </c>
       <c r="F6" s="27">
         <f t="shared" ref="F6:H9" si="0">IFERROR(COUNTIFS($E$14:$E$247,F$5,$H$14:$H$247,$E6),"")</f>
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G6" s="27">
         <f t="shared" si="0"/>
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H6" s="27">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I6" s="16">
         <f>IFERROR(SUM(F6:H6),"-")</f>
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="J6" s="17">
         <f>IFERROR(I6/$I$10,"-")</f>
-        <v>0.91326530612244894</v>
+        <v>0.9441624365482234</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -2396,11 +2399,11 @@
       </c>
       <c r="F7" s="27">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7" s="27">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H7" s="27">
         <f t="shared" si="0"/>
@@ -2408,11 +2411,11 @@
       </c>
       <c r="I7" s="16">
         <f>IFERROR(SUM(F7:H7),"-")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J7" s="17">
         <f>IFERROR(I7/$I$10,"-")</f>
-        <v>3.5714285714285712E-2</v>
+        <v>5.0761421319796954E-2</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -2428,19 +2431,19 @@
       </c>
       <c r="G8" s="27">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H8" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I8" s="16">
         <f>IFERROR(SUM(F8:H8),"-")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J8" s="17">
         <f>IFERROR(I8/$I$10,"-")</f>
-        <v>4.5918367346938778E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
@@ -2468,7 +2471,7 @@
       </c>
       <c r="J9" s="17">
         <f>IFERROR(I9/$I$10,"-")</f>
-        <v>5.1020408163265302E-3</v>
+        <v>5.076142131979695E-3</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
@@ -2486,7 +2489,7 @@
       </c>
       <c r="G10" s="16">
         <f>IFERROR(SUM(G6:G9),"-")</f>
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H10" s="16">
         <f>IFERROR(SUM(H6:H9),"-")</f>
@@ -2494,7 +2497,7 @@
       </c>
       <c r="I10" s="16">
         <f>IFERROR(SUM(F10:H10),"-")</f>
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J10" s="18"/>
     </row>
@@ -2509,15 +2512,15 @@
       </c>
       <c r="F11" s="17">
         <f>IFERROR(F10/$I$10,"-")</f>
-        <v>0.28061224489795916</v>
+        <v>0.27918781725888325</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" ref="G11:H11" si="1">IFERROR(G10/$I$10,"-")</f>
-        <v>0.52551020408163263</v>
+        <v>0.52791878172588835</v>
       </c>
       <c r="H11" s="17">
         <f t="shared" si="1"/>
-        <v>0.19387755102040816</v>
+        <v>0.19289340101522842</v>
       </c>
       <c r="I11" s="18"/>
       <c r="J11" s="19"/>
@@ -6379,7 +6382,7 @@
       <c r="F195" s="24"/>
       <c r="G195" s="24"/>
       <c r="H195" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I195" s="25"/>
       <c r="J195" s="25"/>
@@ -6400,7 +6403,7 @@
       <c r="F196" s="24"/>
       <c r="G196" s="24"/>
       <c r="H196" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I196" s="25"/>
       <c r="J196" s="25"/>
@@ -6421,7 +6424,7 @@
       <c r="F197" s="24"/>
       <c r="G197" s="24"/>
       <c r="H197" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I197" s="25"/>
       <c r="J197" s="25"/>
@@ -6442,7 +6445,7 @@
       <c r="F198" s="24"/>
       <c r="G198" s="24"/>
       <c r="H198" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I198" s="25"/>
       <c r="J198" s="25"/>
@@ -6463,7 +6466,7 @@
       <c r="F199" s="24"/>
       <c r="G199" s="24"/>
       <c r="H199" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I199" s="25"/>
       <c r="J199" s="25"/>
@@ -6484,7 +6487,7 @@
       <c r="F200" s="24"/>
       <c r="G200" s="24"/>
       <c r="H200" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I200" s="25"/>
       <c r="J200" s="25"/>
@@ -6505,7 +6508,7 @@
       <c r="F201" s="24"/>
       <c r="G201" s="24"/>
       <c r="H201" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I201" s="25"/>
       <c r="J201" s="25"/>
@@ -6526,7 +6529,7 @@
       <c r="F202" s="24"/>
       <c r="G202" s="24"/>
       <c r="H202" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I202" s="25"/>
       <c r="J202" s="25"/>
@@ -6547,7 +6550,7 @@
       <c r="F203" s="24"/>
       <c r="G203" s="24"/>
       <c r="H203" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I203" s="25"/>
       <c r="J203" s="25"/>
@@ -6568,7 +6571,7 @@
       <c r="F204" s="24"/>
       <c r="G204" s="24"/>
       <c r="H204" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I204" s="25"/>
       <c r="J204" s="25"/>
@@ -6589,7 +6592,7 @@
       <c r="F205" s="24"/>
       <c r="G205" s="24"/>
       <c r="H205" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I205" s="25"/>
       <c r="J205" s="25"/>
@@ -6610,7 +6613,7 @@
       <c r="F206" s="24"/>
       <c r="G206" s="24"/>
       <c r="H206" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I206" s="25"/>
       <c r="J206" s="25"/>
@@ -6631,7 +6634,7 @@
       <c r="F207" s="24"/>
       <c r="G207" s="24"/>
       <c r="H207" s="24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I207" s="25"/>
       <c r="J207" s="25"/>
@@ -6673,7 +6676,7 @@
       <c r="F209" s="24"/>
       <c r="G209" s="24"/>
       <c r="H209" s="24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I209" s="25"/>
       <c r="J209" s="25"/>
@@ -6694,19 +6697,29 @@
       <c r="F210" s="24"/>
       <c r="G210" s="24"/>
       <c r="H210" s="24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I210" s="25"/>
       <c r="J210" s="25"/>
     </row>
     <row r="211" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B211" s="21"/>
-      <c r="C211" s="22"/>
-      <c r="D211" s="23"/>
-      <c r="E211" s="24"/>
+      <c r="B211" s="21">
+        <v>195</v>
+      </c>
+      <c r="C211" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D211" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="E211" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="F211" s="24"/>
       <c r="G211" s="24"/>
-      <c r="H211" s="24"/>
+      <c r="H211" s="24" t="s">
+        <v>11</v>
+      </c>
       <c r="I211" s="25"/>
       <c r="J211" s="25"/>
     </row>

</xml_diff>